<commit_message>
Maize Commnunity Survey Import file added a row of data from the test run
</commit_message>
<xml_diff>
--- a/data/output/maize_community_survey_import.xlsx
+++ b/data/output/maize_community_survey_import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM5"/>
+  <dimension ref="A1:CM6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2475,6 +2475,339 @@
       <c r="CL5" t="inlineStr"/>
       <c r="CM5" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.0.0.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>R_papertrail_0001</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BL6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BO6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="BQ6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="BT6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BU6" t="inlineStr">
+        <is>
+          <t>5,6</t>
+        </is>
+      </c>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tested a new survey
</commit_message>
<xml_diff>
--- a/data/output/maize_community_survey_import.xlsx
+++ b/data/output/maize_community_survey_import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM3"/>
+  <dimension ref="A1:CM4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1729,6 +1729,227 @@
       <c r="CL3" t="inlineStr"/>
       <c r="CM3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.0.0.0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>R_papertrail_0001</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BL4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BM4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="BQ4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr"/>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
+      <c r="CI4" t="inlineStr"/>
+      <c r="CJ4" t="inlineStr"/>
+      <c r="CK4" t="inlineStr"/>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move test.py files to the test folder
</commit_message>
<xml_diff>
--- a/data/output/maize_community_survey_import.xlsx
+++ b/data/output/maize_community_survey_import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM5"/>
+  <dimension ref="A1:CM6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2159,6 +2159,275 @@
       <c r="CL5" t="inlineStr"/>
       <c r="CM5" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.0.0.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>R_papertrail_0001</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BL6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BO6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="BQ6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>